<commit_message>
feat: add the original data that author used
</commit_message>
<xml_diff>
--- a/NSCLC.xlsx
+++ b/NSCLC.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ebmhealth-my.sharepoint.com/personal/ananda_biswas_ebmhealth_in/Documents/Documents/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F4FD308-0E4E-4AD3-8CEC-CD8E7BD29D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{1F4FD308-0E4E-4AD3-8CEC-CD8E7BD29D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EC8FAC0-2A4A-4E04-ABFD-57EC16242EF4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AgD" sheetId="1" r:id="rId1"/>
-    <sheet name="Description" sheetId="2" r:id="rId2"/>
+    <sheet name="AgD Type 1" sheetId="3" r:id="rId1"/>
+    <sheet name="AgD Type 2" sheetId="1" r:id="rId2"/>
+    <sheet name="Description" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="108">
   <si>
     <r>
       <rPr>
@@ -541,13 +542,180 @@
   </si>
   <si>
     <t>Click here</t>
+  </si>
+  <si>
+    <t>Study</t>
+  </si>
+  <si>
+    <t>HR.OS</t>
+  </si>
+  <si>
+    <t>OS.ln.HR</t>
+  </si>
+  <si>
+    <t>OS.se</t>
+  </si>
+  <si>
+    <t>HR.PFS</t>
+  </si>
+  <si>
+    <t>PFS.ln.HR</t>
+  </si>
+  <si>
+    <t>PFS.se</t>
+  </si>
+  <si>
+    <t>n1</t>
+  </si>
+  <si>
+    <t>n2</t>
+  </si>
+  <si>
+    <t>non.prop</t>
+  </si>
+  <si>
+    <t>Study 1</t>
+  </si>
+  <si>
+    <t>Study 2</t>
+  </si>
+  <si>
+    <t>Study 3</t>
+  </si>
+  <si>
+    <t>Study 4</t>
+  </si>
+  <si>
+    <t>Study 5</t>
+  </si>
+  <si>
+    <t>Study 6</t>
+  </si>
+  <si>
+    <t>Study 7</t>
+  </si>
+  <si>
+    <t>Study 8</t>
+  </si>
+  <si>
+    <t>Study 9</t>
+  </si>
+  <si>
+    <t>Study 10</t>
+  </si>
+  <si>
+    <t>Study 11</t>
+  </si>
+  <si>
+    <t>Study 12</t>
+  </si>
+  <si>
+    <t>Study 13</t>
+  </si>
+  <si>
+    <t>Study 14</t>
+  </si>
+  <si>
+    <t>Study 15</t>
+  </si>
+  <si>
+    <t>Study 16</t>
+  </si>
+  <si>
+    <t>Study 17</t>
+  </si>
+  <si>
+    <t>Study 18</t>
+  </si>
+  <si>
+    <t>Study 19</t>
+  </si>
+  <si>
+    <t>Study 20</t>
+  </si>
+  <si>
+    <t>Study 21</t>
+  </si>
+  <si>
+    <t>Study 22</t>
+  </si>
+  <si>
+    <t>Study 23</t>
+  </si>
+  <si>
+    <t>Study 24</t>
+  </si>
+  <si>
+    <t>Study 25</t>
+  </si>
+  <si>
+    <t>Study 26</t>
+  </si>
+  <si>
+    <t>Study 27</t>
+  </si>
+  <si>
+    <t>Study 28</t>
+  </si>
+  <si>
+    <t>Study 29</t>
+  </si>
+  <si>
+    <t>Study 30</t>
+  </si>
+  <si>
+    <t>Study 31</t>
+  </si>
+  <si>
+    <t>Study 32</t>
+  </si>
+  <si>
+    <t>Study 33</t>
+  </si>
+  <si>
+    <t>Study 34</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">AgD Type 1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Century Schoolbook"/>
+        <family val="1"/>
+      </rPr>
+      <t>is what the author has used for this calculations.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Century Schoolbook"/>
+        <family val="1"/>
+      </rPr>
+      <t>AgD Type 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Century Schoolbook"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> is what the author has provided in the supplementary materials.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -558,10 +726,12 @@
       <b/>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -579,11 +749,6 @@
       <sz val="8"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -627,6 +792,26 @@
       <sz val="12"/>
       <color theme="10"/>
       <name val="Congenial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Century Schoolbook"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Century Schoolbook"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -680,10 +865,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -705,20 +890,27 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1026,6 +1218,1139 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85ED927E-BB87-42F0-9093-02B882884941}">
+  <dimension ref="A1:J35"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="10" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="13">
+        <v>0.74081822068171799</v>
+      </c>
+      <c r="C2" s="13">
+        <v>-0.3</v>
+      </c>
+      <c r="D2" s="13">
+        <v>0.18</v>
+      </c>
+      <c r="E2" s="13">
+        <v>0.72000292822582002</v>
+      </c>
+      <c r="F2" s="13">
+        <v>-0.32850000000000001</v>
+      </c>
+      <c r="G2" s="13">
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="H2" s="13">
+        <v>82</v>
+      </c>
+      <c r="I2" s="13">
+        <v>73</v>
+      </c>
+      <c r="J2" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="13">
+        <v>0.75578374145572502</v>
+      </c>
+      <c r="C3" s="13">
+        <v>-0.28000000000000003</v>
+      </c>
+      <c r="D3" s="13">
+        <v>0.25</v>
+      </c>
+      <c r="E3" s="13">
+        <v>0.91998308037951204</v>
+      </c>
+      <c r="F3" s="13">
+        <v>-8.3400000000000002E-2</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0.255</v>
+      </c>
+      <c r="H3" s="13">
+        <v>34</v>
+      </c>
+      <c r="I3" s="13">
+        <v>42</v>
+      </c>
+      <c r="J3" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="13">
+        <v>1.2769826622243301</v>
+      </c>
+      <c r="C4" s="13">
+        <v>0.2445</v>
+      </c>
+      <c r="D4" s="13">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="E4" s="13">
+        <v>1.11907225691278</v>
+      </c>
+      <c r="F4" s="13">
+        <v>0.1125</v>
+      </c>
+      <c r="G4" s="13">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="H4" s="13">
+        <v>73</v>
+      </c>
+      <c r="I4" s="13">
+        <v>74</v>
+      </c>
+      <c r="J4" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="13">
+        <v>1.0100501670841699</v>
+      </c>
+      <c r="C5" s="13">
+        <v>0.01</v>
+      </c>
+      <c r="D5" s="13">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="E5" s="13">
+        <v>1.30996445073325</v>
+      </c>
+      <c r="F5" s="13">
+        <v>0.27</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0.13400000000000001</v>
+      </c>
+      <c r="H5" s="13">
+        <v>136</v>
+      </c>
+      <c r="I5" s="13">
+        <v>138</v>
+      </c>
+      <c r="J5" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="13">
+        <v>0.42998713041924003</v>
+      </c>
+      <c r="C6" s="13">
+        <v>-0.84399999999999997</v>
+      </c>
+      <c r="D6" s="13">
+        <v>0.189</v>
+      </c>
+      <c r="E6" s="13">
+        <v>0.539992515340732</v>
+      </c>
+      <c r="F6" s="13">
+        <v>-0.61619999999999997</v>
+      </c>
+      <c r="G6" s="13">
+        <v>0.17</v>
+      </c>
+      <c r="H6" s="13">
+        <v>95</v>
+      </c>
+      <c r="I6" s="13">
+        <v>86</v>
+      </c>
+      <c r="J6" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="13">
+        <v>0.69998246097684302</v>
+      </c>
+      <c r="C7" s="13">
+        <v>-0.35670000000000002</v>
+      </c>
+      <c r="D7" s="13">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0.74998655445935902</v>
+      </c>
+      <c r="F7" s="13">
+        <v>-0.28770000000000001</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0.186</v>
+      </c>
+      <c r="H7" s="13">
+        <v>75</v>
+      </c>
+      <c r="I7" s="13">
+        <v>69</v>
+      </c>
+      <c r="J7" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="13">
+        <v>0.52998848451616598</v>
+      </c>
+      <c r="C8" s="13">
+        <v>-0.63490000000000002</v>
+      </c>
+      <c r="D8" s="13">
+        <v>0.26900000000000002</v>
+      </c>
+      <c r="E8" s="13">
+        <v>0.539992515340732</v>
+      </c>
+      <c r="F8" s="13">
+        <v>-0.61619999999999997</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="H8" s="13">
+        <v>42</v>
+      </c>
+      <c r="I8" s="13">
+        <v>39</v>
+      </c>
+      <c r="J8" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="13">
+        <v>1.03634489638182</v>
+      </c>
+      <c r="C9" s="13">
+        <v>3.5700000000000003E-2</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0.126</v>
+      </c>
+      <c r="E9" s="13">
+        <v>1.0118698946483999</v>
+      </c>
+      <c r="F9" s="13">
+        <v>1.18E-2</v>
+      </c>
+      <c r="G9" s="13">
+        <v>0.126</v>
+      </c>
+      <c r="H9" s="13">
+        <v>125</v>
+      </c>
+      <c r="I9" s="13">
+        <v>125</v>
+      </c>
+      <c r="J9" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="13">
+        <v>1.2814599321940201</v>
+      </c>
+      <c r="C10" s="13">
+        <v>0.248</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0.184</v>
+      </c>
+      <c r="E10" s="13">
+        <v>1.3888832403281</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0.32850000000000001</v>
+      </c>
+      <c r="G10" s="13">
+        <v>0.13700000000000001</v>
+      </c>
+      <c r="H10" s="13">
+        <v>109</v>
+      </c>
+      <c r="I10" s="13">
+        <v>110</v>
+      </c>
+      <c r="J10" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="13">
+        <v>0.85727202101145705</v>
+      </c>
+      <c r="C11" s="13">
+        <v>-0.154</v>
+      </c>
+      <c r="D11" s="13">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="E11" s="13">
+        <v>0.76002800324923403</v>
+      </c>
+      <c r="F11" s="13">
+        <v>-0.27439999999999998</v>
+      </c>
+      <c r="G11" s="13">
+        <v>0.06</v>
+      </c>
+      <c r="H11" s="13">
+        <v>622</v>
+      </c>
+      <c r="I11" s="13">
+        <v>618</v>
+      </c>
+      <c r="J11" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="13">
+        <v>1.03045453395352</v>
+      </c>
+      <c r="C12" s="13">
+        <v>0.03</v>
+      </c>
+      <c r="D12" s="13">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="E12" s="13">
+        <v>0.83002455026201405</v>
+      </c>
+      <c r="F12" s="13">
+        <v>-0.18629999999999999</v>
+      </c>
+      <c r="G12" s="13">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="H12" s="13">
+        <v>353</v>
+      </c>
+      <c r="I12" s="13">
+        <v>360</v>
+      </c>
+      <c r="J12" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="13">
+        <v>0.76997286886149097</v>
+      </c>
+      <c r="C13" s="13">
+        <v>-0.26140000000000002</v>
+      </c>
+      <c r="D13" s="13">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="E13" s="13">
+        <v>0.83002455026201405</v>
+      </c>
+      <c r="F13" s="13">
+        <v>-0.18629999999999999</v>
+      </c>
+      <c r="G13" s="13">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="H13" s="13">
+        <v>76</v>
+      </c>
+      <c r="I13" s="13">
+        <v>81</v>
+      </c>
+      <c r="J13" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="13">
+        <v>0.69998246097684302</v>
+      </c>
+      <c r="C14" s="13">
+        <v>-0.35670000000000002</v>
+      </c>
+      <c r="D14" s="13">
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="E14" s="13">
+        <v>0.64998889555494899</v>
+      </c>
+      <c r="F14" s="13">
+        <v>-0.43080000000000002</v>
+      </c>
+      <c r="G14" s="13">
+        <v>0.255</v>
+      </c>
+      <c r="H14" s="13">
+        <v>33</v>
+      </c>
+      <c r="I14" s="13">
+        <v>35</v>
+      </c>
+      <c r="J14" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="13">
+        <v>0.99800199866733297</v>
+      </c>
+      <c r="C15" s="13">
+        <v>-2E-3</v>
+      </c>
+      <c r="D15" s="13">
+        <v>0.129</v>
+      </c>
+      <c r="E15" s="13">
+        <v>1.24135062430017</v>
+      </c>
+      <c r="F15" s="13">
+        <v>0.2162</v>
+      </c>
+      <c r="G15" s="13">
+        <v>0.11</v>
+      </c>
+      <c r="H15" s="13">
+        <v>166</v>
+      </c>
+      <c r="I15" s="13">
+        <v>166</v>
+      </c>
+      <c r="J15" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="13">
+        <v>1.02757329687277</v>
+      </c>
+      <c r="C16" s="13">
+        <v>2.7199999999999998E-2</v>
+      </c>
+      <c r="D16" s="13">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="E16" s="13">
+        <v>0.77159151086535305</v>
+      </c>
+      <c r="F16" s="13">
+        <v>-0.25929999999999997</v>
+      </c>
+      <c r="G16" s="13">
+        <v>0.29099999999999998</v>
+      </c>
+      <c r="H16" s="13">
+        <v>26</v>
+      </c>
+      <c r="I16" s="13">
+        <v>24</v>
+      </c>
+      <c r="J16" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="13">
+        <v>0.83326796655878499</v>
+      </c>
+      <c r="C17" s="13">
+        <v>-0.18240000000000001</v>
+      </c>
+      <c r="D17" s="13">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="E17" s="13">
+        <v>0.91283512561622304</v>
+      </c>
+      <c r="F17" s="13">
+        <v>-9.1200000000000003E-2</v>
+      </c>
+      <c r="G17" s="13">
+        <v>0.157</v>
+      </c>
+      <c r="H17" s="13">
+        <v>99</v>
+      </c>
+      <c r="I17" s="13">
+        <v>102</v>
+      </c>
+      <c r="J17" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" s="13">
+        <v>2.03663716675063</v>
+      </c>
+      <c r="C18" s="13">
+        <v>0.71130000000000004</v>
+      </c>
+      <c r="D18" s="13">
+        <v>0.245</v>
+      </c>
+      <c r="E18" s="13">
+        <v>2.8662369437164599</v>
+      </c>
+      <c r="F18" s="13">
+        <v>1.0529999999999999</v>
+      </c>
+      <c r="G18" s="13">
+        <v>0.23499999999999999</v>
+      </c>
+      <c r="H18" s="13">
+        <v>26</v>
+      </c>
+      <c r="I18" s="13">
+        <v>102</v>
+      </c>
+      <c r="J18" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="13">
+        <v>0.42037840880178201</v>
+      </c>
+      <c r="C19" s="13">
+        <v>-0.86660000000000004</v>
+      </c>
+      <c r="D19" s="13">
+        <v>0.255</v>
+      </c>
+      <c r="E19" s="13">
+        <v>0.20341643444169</v>
+      </c>
+      <c r="F19" s="13">
+        <v>-1.5925</v>
+      </c>
+      <c r="G19" s="13">
+        <v>0.249</v>
+      </c>
+      <c r="H19" s="13">
+        <v>99</v>
+      </c>
+      <c r="I19" s="13">
+        <v>24</v>
+      </c>
+      <c r="J19" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="13">
+        <v>1.0988893632810799</v>
+      </c>
+      <c r="C20" s="13">
+        <v>9.4299999999999995E-2</v>
+      </c>
+      <c r="D20" s="13">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="E20" s="13">
+        <v>0.81963185242014502</v>
+      </c>
+      <c r="F20" s="13">
+        <v>-0.19889999999999999</v>
+      </c>
+      <c r="G20" s="13">
+        <v>0.12</v>
+      </c>
+      <c r="H20" s="13">
+        <v>151</v>
+      </c>
+      <c r="I20" s="13">
+        <v>150</v>
+      </c>
+      <c r="J20" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="13">
+        <v>1.02020134002676</v>
+      </c>
+      <c r="C21" s="13">
+        <v>0.02</v>
+      </c>
+      <c r="D21" s="13">
+        <v>0.06</v>
+      </c>
+      <c r="E21" s="13">
+        <v>1.03997845854368</v>
+      </c>
+      <c r="F21" s="13">
+        <v>3.9199999999999999E-2</v>
+      </c>
+      <c r="G21" s="13">
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="H21" s="13">
+        <v>723</v>
+      </c>
+      <c r="I21" s="13">
+        <v>710</v>
+      </c>
+      <c r="J21" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" s="13">
+        <v>1</v>
+      </c>
+      <c r="C22" s="13">
+        <v>0</v>
+      </c>
+      <c r="D22" s="13">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="E22" s="13">
+        <v>1</v>
+      </c>
+      <c r="F22" s="13">
+        <v>0</v>
+      </c>
+      <c r="G22" s="13">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="H22" s="13">
+        <v>45</v>
+      </c>
+      <c r="I22" s="13">
+        <v>43</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B23" s="13">
+        <v>1.44051400814922</v>
+      </c>
+      <c r="C23" s="13">
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="D23" s="13">
+        <v>0.218</v>
+      </c>
+      <c r="E23" s="13">
+        <v>0.989950833715877</v>
+      </c>
+      <c r="F23" s="13">
+        <v>-1.01E-2</v>
+      </c>
+      <c r="G23" s="13">
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="H23" s="13">
+        <v>77</v>
+      </c>
+      <c r="I23" s="13">
+        <v>82</v>
+      </c>
+      <c r="J23" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B24" s="13">
+        <v>1.0800420763926</v>
+      </c>
+      <c r="C24" s="13">
+        <v>7.6999999999999999E-2</v>
+      </c>
+      <c r="D24" s="13">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="E24" s="13">
+        <v>0.57001078344952005</v>
+      </c>
+      <c r="F24" s="13">
+        <v>-0.56210000000000004</v>
+      </c>
+      <c r="G24" s="13">
+        <v>0.18</v>
+      </c>
+      <c r="H24" s="13">
+        <v>75</v>
+      </c>
+      <c r="I24" s="13">
+        <v>82</v>
+      </c>
+      <c r="J24" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" s="13">
+        <v>0.74976159223904104</v>
+      </c>
+      <c r="C25" s="13">
+        <v>-0.28799999999999998</v>
+      </c>
+      <c r="D25" s="13">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="E25" s="13">
+        <v>0.580015761970338</v>
+      </c>
+      <c r="F25" s="13">
+        <v>-0.54469999999999996</v>
+      </c>
+      <c r="G25" s="13">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="H25" s="13">
+        <v>75</v>
+      </c>
+      <c r="I25" s="13">
+        <v>77</v>
+      </c>
+      <c r="J25" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="13">
+        <v>0.76997286886149097</v>
+      </c>
+      <c r="C26" s="13">
+        <v>-0.26140000000000002</v>
+      </c>
+      <c r="D26" s="13">
+        <v>0.32</v>
+      </c>
+      <c r="E26" s="13">
+        <v>0.63002233994191204</v>
+      </c>
+      <c r="F26" s="13">
+        <v>-0.46200000000000002</v>
+      </c>
+      <c r="G26" s="13">
+        <v>0.25800000000000001</v>
+      </c>
+      <c r="H26" s="13">
+        <v>31</v>
+      </c>
+      <c r="I26" s="13">
+        <v>21</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" s="13">
+        <v>0.80003484181006601</v>
+      </c>
+      <c r="C27" s="13">
+        <v>-0.22309999999999999</v>
+      </c>
+      <c r="D27" s="13">
+        <v>0.27400000000000002</v>
+      </c>
+      <c r="E27" s="13">
+        <v>1.19053168326383</v>
+      </c>
+      <c r="F27" s="13">
+        <v>0.1744</v>
+      </c>
+      <c r="G27" s="13">
+        <v>0.23499999999999999</v>
+      </c>
+      <c r="H27" s="13">
+        <v>45</v>
+      </c>
+      <c r="I27" s="13">
+        <v>45</v>
+      </c>
+      <c r="J27" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="13">
+        <v>0.83027359498193298</v>
+      </c>
+      <c r="C28" s="13">
+        <v>-0.186</v>
+      </c>
+      <c r="D28" s="13">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="E28" s="13">
+        <v>0.76997286886149097</v>
+      </c>
+      <c r="F28" s="13">
+        <v>-0.26140000000000002</v>
+      </c>
+      <c r="G28" s="13">
+        <v>0.112</v>
+      </c>
+      <c r="H28" s="13">
+        <v>322</v>
+      </c>
+      <c r="I28" s="13">
+        <v>336</v>
+      </c>
+      <c r="J28" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" s="13">
+        <v>1.0100501670841699</v>
+      </c>
+      <c r="C29" s="13">
+        <v>0.01</v>
+      </c>
+      <c r="D29" s="13">
+        <v>0.09</v>
+      </c>
+      <c r="E29" s="13">
+        <v>0.76997286886149097</v>
+      </c>
+      <c r="F29" s="13">
+        <v>-0.26140000000000002</v>
+      </c>
+      <c r="G29" s="13">
+        <v>0.112</v>
+      </c>
+      <c r="H29" s="13">
+        <v>276</v>
+      </c>
+      <c r="I29" s="13">
+        <v>279</v>
+      </c>
+      <c r="J29" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B30" s="13">
+        <v>0.78035994327803404</v>
+      </c>
+      <c r="C30" s="13">
+        <v>-0.248</v>
+      </c>
+      <c r="D30" s="13">
+        <v>0.126</v>
+      </c>
+      <c r="E30" s="13">
+        <v>0.81995977074040505</v>
+      </c>
+      <c r="F30" s="13">
+        <v>-0.19850000000000001</v>
+      </c>
+      <c r="G30" s="13">
+        <v>0.111</v>
+      </c>
+      <c r="H30" s="13">
+        <v>205</v>
+      </c>
+      <c r="I30" s="13">
+        <v>194</v>
+      </c>
+      <c r="J30" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" s="13">
+        <v>1.56049019583267</v>
+      </c>
+      <c r="C31" s="13">
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="D31" s="13">
+        <v>0.188</v>
+      </c>
+      <c r="E31" s="13">
+        <v>1.40003886926987</v>
+      </c>
+      <c r="F31" s="13">
+        <v>0.33650000000000002</v>
+      </c>
+      <c r="G31" s="13">
+        <v>0.16900000000000001</v>
+      </c>
+      <c r="H31" s="13">
+        <v>78</v>
+      </c>
+      <c r="I31" s="13">
+        <v>94</v>
+      </c>
+      <c r="J31" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="13">
+        <v>1.2460767305873801</v>
+      </c>
+      <c r="C32" s="13">
+        <v>0.22</v>
+      </c>
+      <c r="D32" s="13">
+        <v>0.24</v>
+      </c>
+      <c r="E32" s="13">
+        <v>1.8518775197634101</v>
+      </c>
+      <c r="F32" s="13">
+        <v>0.61619999999999997</v>
+      </c>
+      <c r="G32" s="13">
+        <v>0.19400000000000001</v>
+      </c>
+      <c r="H32" s="13">
+        <v>67</v>
+      </c>
+      <c r="I32" s="13">
+        <v>68</v>
+      </c>
+      <c r="J32" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="13">
+        <v>1.02020134002676</v>
+      </c>
+      <c r="C33" s="13">
+        <v>0.02</v>
+      </c>
+      <c r="D33" s="13">
+        <v>0.16300000000000001</v>
+      </c>
+      <c r="E33" s="13">
+        <v>1.05001032767289</v>
+      </c>
+      <c r="F33" s="13">
+        <v>4.8800000000000003E-2</v>
+      </c>
+      <c r="G33" s="13">
+        <v>0.17</v>
+      </c>
+      <c r="H33" s="13">
+        <v>104</v>
+      </c>
+      <c r="I33" s="13">
+        <v>98</v>
+      </c>
+      <c r="J33" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B34" s="13">
+        <v>0.74000376866969897</v>
+      </c>
+      <c r="C34" s="13">
+        <v>-0.30109999999999998</v>
+      </c>
+      <c r="D34" s="13">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="E34" s="13">
+        <v>0.70999311938555099</v>
+      </c>
+      <c r="F34" s="13">
+        <v>-0.34250000000000003</v>
+      </c>
+      <c r="G34" s="13">
+        <v>0.215</v>
+      </c>
+      <c r="H34" s="13">
+        <v>50</v>
+      </c>
+      <c r="I34" s="13">
+        <v>50</v>
+      </c>
+      <c r="J34" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B35" s="13">
+        <v>0.71892373343192595</v>
+      </c>
+      <c r="C35" s="13">
+        <v>-0.33</v>
+      </c>
+      <c r="D35" s="13">
+        <v>0.19</v>
+      </c>
+      <c r="E35" s="13">
+        <v>0.52998848451616598</v>
+      </c>
+      <c r="F35" s="13">
+        <v>-0.63490000000000002</v>
+      </c>
+      <c r="G35" s="13">
+        <v>0.17299999999999999</v>
+      </c>
+      <c r="H35" s="13">
+        <v>76</v>
+      </c>
+      <c r="I35" s="13">
+        <v>81</v>
+      </c>
+      <c r="J35" s="13">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K35"/>
   <sheetFormatPr defaultColWidth="9.296875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
@@ -2273,12 +3598,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDD26A89-69C8-4EB1-B8F9-929B7F6DEC83}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="54.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="96.796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2287,7 +3612,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="21.5" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>58</v>
       </c>
@@ -2351,9 +3676,23 @@
         <v>61</v>
       </c>
     </row>
+    <row r="19" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A19" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
+        <v>107</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B14" r:id="rId1" xr:uid="{B90A80EC-BDFF-4556-9C19-E0F0BAF7517D}"/>
+    <hyperlink ref="B19" r:id="rId2" xr:uid="{57E47DDF-70C1-418F-B4D0-1866FFB05DA8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>